<commit_message>
Added couple of new code changes
</commit_message>
<xml_diff>
--- a/SalamtekAppiumAndroid/src/test/resources/TestData/TestDataAndroid.xlsx
+++ b/SalamtekAppiumAndroid/src/test/resources/TestData/TestDataAndroid.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.barried\git\Salamtek_Website\SalamtekAppiumAndroid\src\test\resources\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.barried\git\Salamtek_Android_v1\SalamtekAppiumAndroid\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C6ADCE-B0A8-4632-A996-8F45BCA217AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{404AA8DB-92D9-4749-9EA5-691188D70AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BA93E413-0FBB-4423-B223-0A6D5A2FA904}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{BA93E413-0FBB-4423-B223-0A6D5A2FA904}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="3" r:id="rId1"/>
@@ -28,7 +28,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="332">
   <si>
     <t>TestCaseName</t>
   </si>
@@ -757,9 +757,6 @@
     <t>Delivery</t>
   </si>
   <si>
-    <t>Pregnancy belt-M-Black</t>
-  </si>
-  <si>
     <t>SLMTK_T264</t>
   </si>
   <si>
@@ -919,172 +916,144 @@
     <t>Fortis Lab</t>
   </si>
   <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>53</t>
+    <t>Vitamins &amp; Supplements</t>
   </si>
   <si>
     <t>PASS</t>
   </si>
   <si>
-    <t>#200010259</t>
-  </si>
-  <si>
-    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010259 scheduled on 2025-10-19 at 11:45 am.</t>
-  </si>
-  <si>
-    <t>#300006421</t>
-  </si>
-  <si>
-    <t>You have booked an appointment #300006421 at Hitech Lab</t>
-  </si>
-  <si>
-    <t>#300006422</t>
-  </si>
-  <si>
-    <t>You have rescheduled your appointment #300006422 at Hitech Lab</t>
-  </si>
-  <si>
-    <t>#300006423</t>
+    <t>#200010517</t>
+  </si>
+  <si>
+    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010517 scheduled on 2026-01-25 at 01:45 pm.</t>
+  </si>
+  <si>
+    <t>#300006505</t>
+  </si>
+  <si>
+    <t>You have booked an appointment #300006505 at Hitech Lab</t>
+  </si>
+  <si>
+    <t>#300006506</t>
+  </si>
+  <si>
+    <t>Your appointment has been cancelled successfully. 
+ Your refund amount is KD 10.000</t>
+  </si>
+  <si>
+    <t>You have cancelled your lab appointment #300006506 at Hitech Lab</t>
+  </si>
+  <si>
+    <t>#100006199</t>
+  </si>
+  <si>
+    <t>You have placed an order#100006199 at Health Is Wealth</t>
+  </si>
+  <si>
+    <t>#100006200</t>
+  </si>
+  <si>
+    <t>Order Cancelled Successfully. 
+ Your refund amount is KD 25.000</t>
+  </si>
+  <si>
+    <t>You cancelled an order #100006200 at Health Is Wealth</t>
+  </si>
+  <si>
+    <t>Digene</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Pregnancy belt</t>
+  </si>
+  <si>
+    <t>#200010551</t>
+  </si>
+  <si>
+    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010551 scheduled on 2026-01-28 at 11:00 am.</t>
+  </si>
+  <si>
+    <t>#200010552</t>
+  </si>
+  <si>
+    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010552 scheduled on 2026-01-28 at 11:15 am.</t>
+  </si>
+  <si>
+    <t>#200010554</t>
+  </si>
+  <si>
+    <t>You have successfully rescheduled a doctor appointment #200010554 with Livana Clarus Linto</t>
+  </si>
+  <si>
+    <t>#200010555</t>
+  </si>
+  <si>
+    <t>Your appointment has been cancelled successfully. 
+ Your refund amount is KD 13.000</t>
+  </si>
+  <si>
+    <t>You have cancelled a doctor appointment #200010555 with Livana Clarus Linto</t>
+  </si>
+  <si>
+    <t>#200010556</t>
   </si>
   <si>
     <t>Your appointment has been cancelled successfully. 
  Your refunded amount will be processed and returned to your bank account within 5 to 7 business days.</t>
   </si>
   <si>
-    <t>You have cancelled your lab appointment #300006423 at Hitech Lab</t>
-  </si>
-  <si>
-    <t>#300006424</t>
-  </si>
-  <si>
-    <t>Your appointment has been cancelled successfully. 
- Your refund amount is KD 10.000</t>
-  </si>
-  <si>
-    <t>You have cancelled your lab appointment #300006424 at Hitech Lab</t>
-  </si>
-  <si>
-    <t>#100006089</t>
-  </si>
-  <si>
-    <t>You have placed an order#100006089 at Health Is Wealth</t>
-  </si>
-  <si>
-    <t>#100006090</t>
-  </si>
-  <si>
-    <t>You have placed an order#100006090 at Health Is Wealth</t>
-  </si>
-  <si>
-    <t>#100006091</t>
-  </si>
-  <si>
-    <t>Order Cancelled Successfully. 
- Your refund amount is KD 25.000</t>
-  </si>
-  <si>
-    <t>You cancelled an order #100006091 at Health Is Wealth</t>
-  </si>
-  <si>
-    <t>Vitamins &amp; Supplements</t>
-  </si>
-  <si>
-    <t>Flamingo Orthopedic Heat Belt</t>
-  </si>
-  <si>
-    <t>#100006092</t>
-  </si>
-  <si>
-    <t>You have placed an order#100006092 at Health Is Wealth</t>
-  </si>
-  <si>
-    <t>#200010263</t>
-  </si>
-  <si>
-    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010263 scheduled on 2025-10-19 at 02:15 pm.</t>
-  </si>
-  <si>
-    <t>#200010264</t>
-  </si>
-  <si>
-    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010264 scheduled on 2025-10-19 at 02:30 pm.</t>
-  </si>
-  <si>
-    <t>#200010266</t>
-  </si>
-  <si>
-    <t>You have successfully rescheduled a doctor appointment #200010266 with Livana Clarus Linto</t>
-  </si>
-  <si>
-    <t>#200010267</t>
-  </si>
-  <si>
-    <t>Your appointment has been cancelled successfully. 
- Your refund amount is KD 13.000</t>
-  </si>
-  <si>
-    <t>You have cancelled a doctor appointment #200010267 with Livana Clarus Linto</t>
-  </si>
-  <si>
-    <t>#100006093</t>
-  </si>
-  <si>
-    <t>You have placed an order#100006093 at Health Is Wealth</t>
-  </si>
-  <si>
-    <t>#100006094</t>
+    <t>You have cancelled a doctor appointment #200010556 with Livana Clarus Linto</t>
+  </si>
+  <si>
+    <t>#300006508</t>
+  </si>
+  <si>
+    <t>You have rescheduled your appointment #300006508 at Hitech Lab</t>
+  </si>
+  <si>
+    <t>#300006509</t>
+  </si>
+  <si>
+    <t>You have cancelled your lab appointment #300006509 at Hitech Lab</t>
+  </si>
+  <si>
+    <t>#100006207</t>
+  </si>
+  <si>
+    <t>You have placed an order#100006207 at Health Is Wealth</t>
+  </si>
+  <si>
+    <t>#100006208</t>
+  </si>
+  <si>
+    <t>You have placed an order#100006208 at Health Is Wealth</t>
+  </si>
+  <si>
+    <t>#100006210</t>
+  </si>
+  <si>
+    <t>You have placed an order#100006210 at Health Is Wealth</t>
+  </si>
+  <si>
+    <t>#100006211</t>
   </si>
   <si>
     <t>Order Cancelled Successfully. 
  Your refunded amount will be processed and returned to your bank account within 5 to 7 business days.</t>
   </si>
   <si>
-    <t>You cancelled an order #100006094 at Health Is Wealth</t>
-  </si>
-  <si>
-    <t>#200010270</t>
-  </si>
-  <si>
-    <t>You have cancelled a doctor appointment #200010270 with Livana Clarus Linto</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>#200010303</t>
-  </si>
-  <si>
-    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010303 scheduled on 2025-11-24 at 01:00 pm.</t>
-  </si>
-  <si>
-    <t>#200010304</t>
-  </si>
-  <si>
-    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010304 scheduled on 2025-11-24 at 01:15 pm.</t>
-  </si>
-  <si>
-    <t>#200010318</t>
-  </si>
-  <si>
-    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010318 scheduled on 2025-11-26 at 12:30 pm.</t>
-  </si>
-  <si>
-    <t>#200010319</t>
-  </si>
-  <si>
-    <t>You have booked a doctor appointment with Livana Clarus Linto. The appointment number is #200010319 scheduled on 2025-11-26 at 02:00 pm.</t>
+    <t>You cancelled an order #100006211 at Health Is Wealth</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1799,12 +1768,12 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="13.0" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="41.0" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="47.5546875" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" width="25.6640625" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="21.109375" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.109375" collapsed="true"/>
+    <col min="1" max="1" width="13" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="41" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="47.5546875" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="25.6640625" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -1831,7 +1800,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1849,8 +1818,8 @@
       <c r="F2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G2" t="s" s="0">
-        <v>292</v>
+      <c r="G2" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -1870,27 +1839,27 @@
   <dimension ref="A1:AK7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="11.109375" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="41.0" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="85.0" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" width="25.6640625" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="21.109375" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.109375" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="16.33203125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="16.88671875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="19.33203125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="20.0"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="12.88671875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="52.33203125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="11.109375"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="13.33203125"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="14.33203125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="15.6640625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="21.88671875"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="78.5546875"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" width="130.109375"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="11.0"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="41" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="85" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="25.6640625" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="52.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="78.5546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="130.109375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.3">
@@ -2007,7 +1976,7 @@
       </c>
     </row>
     <row r="2" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>59</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -2028,7 +1997,6 @@
       <c r="G2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H2" s="0"/>
       <c r="I2" s="3" t="s">
         <v>36</v>
       </c>
@@ -2044,39 +2012,18 @@
       <c r="M2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="N2" s="0"/>
-      <c r="O2" s="0"/>
-      <c r="P2" s="0"/>
-      <c r="Q2" s="0"/>
-      <c r="R2" s="0"/>
-      <c r="S2" s="0"/>
-      <c r="T2" s="0"/>
-      <c r="U2" s="0"/>
-      <c r="V2" s="0"/>
-      <c r="W2" s="0"/>
-      <c r="X2" s="0"/>
-      <c r="Y2" s="0"/>
-      <c r="Z2" s="0"/>
-      <c r="AA2" s="0"/>
-      <c r="AB2" s="0"/>
-      <c r="AC2" s="0"/>
-      <c r="AD2" s="0"/>
-      <c r="AE2" s="0"/>
-      <c r="AF2" s="0"/>
-      <c r="AG2" s="0"/>
-      <c r="AH2" s="0"/>
-      <c r="AI2" t="s" s="0">
-        <v>319</v>
-      </c>
-      <c r="AJ2" t="s" s="0">
-        <v>318</v>
-      </c>
-      <c r="AK2" t="s" s="0">
+      <c r="AI2" t="s">
         <v>292</v>
       </c>
+      <c r="AJ2" t="s">
+        <v>291</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="3" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>60</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -2097,7 +2044,6 @@
       <c r="G3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="0"/>
       <c r="I3" s="3" t="s">
         <v>36</v>
       </c>
@@ -2113,7 +2059,6 @@
       <c r="M3" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="N3" s="0"/>
       <c r="O3" s="2" t="s">
         <v>49</v>
       </c>
@@ -2130,42 +2075,32 @@
         <v>52</v>
       </c>
       <c r="T3" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="U3" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="V3" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="V3" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="W3" s="3" t="s">
         <v>53</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="Y3" s="0"/>
-      <c r="Z3" s="0"/>
-      <c r="AA3" s="0"/>
-      <c r="AB3" s="0"/>
-      <c r="AC3" s="0"/>
-      <c r="AD3" s="0"/>
-      <c r="AE3" s="0"/>
-      <c r="AF3" s="0"/>
-      <c r="AG3" s="0"/>
-      <c r="AH3" s="0"/>
-      <c r="AI3" t="s" s="0">
-        <v>294</v>
-      </c>
-      <c r="AJ3" t="s" s="0">
-        <v>293</v>
-      </c>
-      <c r="AK3" t="s" s="0">
-        <v>292</v>
+        <v>284</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>310</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>309</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>61</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -2175,7 +2110,7 @@
         <v>47</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>332</v>
+        <v>65</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>34</v>
@@ -2186,7 +2121,6 @@
       <c r="G4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="0"/>
       <c r="I4" s="3" t="s">
         <v>36</v>
       </c>
@@ -2205,11 +2139,6 @@
       <c r="N4" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="O4" s="0"/>
-      <c r="P4" s="0"/>
-      <c r="Q4" s="0"/>
-      <c r="R4" s="0"/>
-      <c r="S4" s="0"/>
       <c r="T4" s="3" t="s">
         <v>41</v>
       </c>
@@ -2217,34 +2146,23 @@
         <v>46</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="W4" s="0"/>
-      <c r="X4" s="0"/>
+        <v>287</v>
+      </c>
       <c r="Y4" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="Z4" s="0"/>
-      <c r="AA4" s="0"/>
-      <c r="AB4" s="0"/>
-      <c r="AC4" s="0"/>
-      <c r="AD4" s="0"/>
-      <c r="AE4" s="0"/>
-      <c r="AF4" s="0"/>
-      <c r="AG4" s="0"/>
-      <c r="AH4" s="0"/>
-      <c r="AI4" t="s" s="0">
-        <v>341</v>
-      </c>
-      <c r="AJ4" t="s" s="0">
-        <v>340</v>
-      </c>
-      <c r="AK4" t="s" s="0">
-        <v>292</v>
+      <c r="AI4" t="s">
+        <v>308</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>307</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>64</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -2265,7 +2183,6 @@
       <c r="G5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="0"/>
       <c r="I5" s="3" t="s">
         <v>36</v>
       </c>
@@ -2284,11 +2201,6 @@
       <c r="N5" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="O5" s="0"/>
-      <c r="P5" s="0"/>
-      <c r="Q5" s="0"/>
-      <c r="R5" s="0"/>
-      <c r="S5" s="0"/>
       <c r="T5" s="3" t="s">
         <v>41</v>
       </c>
@@ -2296,34 +2208,23 @@
         <v>46</v>
       </c>
       <c r="V5" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="W5" s="0"/>
-      <c r="X5" s="0"/>
+        <v>287</v>
+      </c>
       <c r="Y5" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="Z5" s="0"/>
-      <c r="AA5" s="0"/>
-      <c r="AB5" s="0"/>
-      <c r="AC5" s="0"/>
-      <c r="AD5" s="0"/>
-      <c r="AE5" s="0"/>
-      <c r="AF5" s="0"/>
-      <c r="AG5" s="0"/>
-      <c r="AH5" s="0"/>
-      <c r="AI5" t="s" s="0">
-        <v>321</v>
-      </c>
-      <c r="AJ5" t="s" s="0">
-        <v>320</v>
-      </c>
-      <c r="AK5" t="s" s="0">
-        <v>292</v>
+      <c r="AI5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>311</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>88</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -2344,7 +2245,6 @@
       <c r="G6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H6" s="0"/>
       <c r="I6" s="3" t="s">
         <v>36</v>
       </c>
@@ -2360,47 +2260,30 @@
       <c r="M6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="N6" s="0"/>
-      <c r="O6" s="0"/>
-      <c r="P6" s="0"/>
-      <c r="Q6" s="0"/>
-      <c r="R6" s="0"/>
-      <c r="S6" s="0"/>
-      <c r="T6" s="0"/>
-      <c r="U6" s="0"/>
-      <c r="V6" s="0"/>
-      <c r="W6" s="0"/>
-      <c r="X6" s="0"/>
-      <c r="Y6" s="0"/>
-      <c r="Z6" s="0"/>
-      <c r="AA6" s="0"/>
-      <c r="AB6" s="0"/>
-      <c r="AC6" s="0"/>
-      <c r="AD6" s="0"/>
-      <c r="AE6" s="0">
+      <c r="AE6">
         <v>13</v>
       </c>
-      <c r="AF6" s="0">
-        <v>1903.2750000000001</v>
-      </c>
-      <c r="AG6" s="0">
-        <v>1901.2750000000001</v>
-      </c>
-      <c r="AH6" t="s" s="0">
-        <v>323</v>
-      </c>
-      <c r="AI6" t="s" s="0">
-        <v>324</v>
-      </c>
-      <c r="AJ6" t="s" s="0">
-        <v>322</v>
-      </c>
-      <c r="AK6" t="s" s="0">
-        <v>292</v>
+      <c r="AF6">
+        <v>2415.2469999999998</v>
+      </c>
+      <c r="AG6">
+        <v>2413.2469999999998</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>314</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>315</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>313</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>84</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -2421,7 +2304,6 @@
       <c r="G7" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="0"/>
       <c r="I7" s="3" t="s">
         <v>36</v>
       </c>
@@ -2440,11 +2322,6 @@
       <c r="N7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="O7" s="0"/>
-      <c r="P7" s="0"/>
-      <c r="Q7" s="0"/>
-      <c r="R7" s="0"/>
-      <c r="S7" s="0"/>
       <c r="T7" s="3" t="s">
         <v>41</v>
       </c>
@@ -2452,32 +2329,22 @@
         <v>46</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="W7" s="0"/>
-      <c r="X7" s="0"/>
+        <v>287</v>
+      </c>
       <c r="Y7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="Z7" s="0"/>
-      <c r="AA7" s="0"/>
-      <c r="AB7" s="0"/>
-      <c r="AC7" s="0"/>
-      <c r="AD7" s="0"/>
-      <c r="AE7" s="0"/>
-      <c r="AF7" s="0"/>
-      <c r="AG7" s="0"/>
-      <c r="AH7" t="s" s="0">
-        <v>300</v>
-      </c>
-      <c r="AI7" t="s" s="0">
-        <v>331</v>
-      </c>
-      <c r="AJ7" t="s" s="0">
-        <v>330</v>
-      </c>
-      <c r="AK7" t="s" s="0">
-        <v>292</v>
+      <c r="AH7" t="s">
+        <v>317</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>318</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>316</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -2523,27 +2390,27 @@
   <dimension ref="A1:AM15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="14.5546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="41.88671875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="84.6640625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="21.109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.109375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="20.0"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="26.109375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="20.0"/>
-    <col min="11" max="11" customWidth="true" width="20.0"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="28.44140625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="10.44140625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="16.5546875"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="16.44140625"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="11.44140625"/>
-    <col min="32" max="32" customWidth="true" width="11.44140625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="14.33203125"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="15.6640625"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" width="21.88671875"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="143.44140625"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" width="64.0"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" width="11.0"/>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="84.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="28.44140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.44140625" customWidth="1"/>
+    <col min="33" max="33" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="143.44140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="64" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" x14ac:dyDescent="0.3">
@@ -2688,7 +2555,7 @@
         <v>77</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>142</v>
@@ -2705,14 +2572,14 @@
       <c r="N2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AK2" t="s" s="0">
-        <v>296</v>
-      </c>
-      <c r="AL2" t="s" s="0">
-        <v>295</v>
-      </c>
-      <c r="AM2" t="s" s="0">
-        <v>292</v>
+      <c r="AK2" t="s">
+        <v>294</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>293</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:39" x14ac:dyDescent="0.3">
@@ -2738,7 +2605,7 @@
         <v>77</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>142</v>
@@ -2771,28 +2638,28 @@
         <v>52</v>
       </c>
       <c r="U3" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="V3" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="V3" s="3" t="s">
+      <c r="W3" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="X3" s="3" t="s">
         <v>53</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="AK3" t="s" s="0">
-        <v>298</v>
-      </c>
-      <c r="AL3" t="s" s="0">
-        <v>297</v>
-      </c>
-      <c r="AM3" t="s" s="0">
-        <v>292</v>
+        <v>284</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>320</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>319</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:39" x14ac:dyDescent="0.3">
@@ -2818,7 +2685,7 @@
         <v>77</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>142</v>
@@ -2851,31 +2718,31 @@
         <v>52</v>
       </c>
       <c r="U4" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="V4" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="V4" s="3" t="s">
+      <c r="W4" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="W4" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="X4" s="3" t="s">
         <v>53</v>
       </c>
       <c r="Y4" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="AJ4" t="s" s="0">
-        <v>300</v>
-      </c>
-      <c r="AK4" t="s" s="0">
-        <v>301</v>
-      </c>
-      <c r="AL4" t="s" s="0">
-        <v>299</v>
-      </c>
-      <c r="AM4" t="s" s="0">
-        <v>292</v>
+        <v>284</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>317</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>322</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>321</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:39" x14ac:dyDescent="0.3">
@@ -2901,7 +2768,7 @@
         <v>77</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>142</v>
@@ -2918,26 +2785,26 @@
       <c r="N5" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AG5" s="0">
+      <c r="AG5">
         <v>10</v>
       </c>
-      <c r="AH5" s="0">
-        <v>1943.2750000000001</v>
-      </c>
-      <c r="AI5" s="0">
-        <v>1943.2750000000001</v>
-      </c>
-      <c r="AJ5" t="s" s="0">
-        <v>303</v>
-      </c>
-      <c r="AK5" t="s" s="0">
-        <v>304</v>
-      </c>
-      <c r="AL5" t="s" s="0">
-        <v>302</v>
-      </c>
-      <c r="AM5" t="s" s="0">
-        <v>292</v>
+      <c r="AH5">
+        <v>2522.2469999999998</v>
+      </c>
+      <c r="AI5">
+        <v>2522.2469999999998</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>296</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>297</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>295</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:39" x14ac:dyDescent="0.3">
@@ -2962,8 +2829,8 @@
       <c r="G6" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="AM6" t="s" s="0">
-        <v>292</v>
+      <c r="AM6" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:39" x14ac:dyDescent="0.3">
@@ -2997,8 +2864,8 @@
       <c r="AD7" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="AM7" t="s" s="0">
-        <v>292</v>
+      <c r="AM7" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.3">
@@ -3032,8 +2899,8 @@
       <c r="AD8" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="AM8" t="s" s="0">
-        <v>292</v>
+      <c r="AM8" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.3">
@@ -3067,8 +2934,8 @@
       <c r="AD9" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="AM9" t="s" s="0">
-        <v>292</v>
+      <c r="AM9" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.3">
@@ -3102,8 +2969,8 @@
       <c r="AD10" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="AM10" t="s" s="0">
-        <v>292</v>
+      <c r="AM10" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.3">
@@ -3135,10 +3002,10 @@
         <v>178</v>
       </c>
       <c r="AD11" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="AM11" t="s" s="0">
-        <v>292</v>
+        <v>288</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="12" spans="1:39" x14ac:dyDescent="0.3">
@@ -3172,16 +3039,16 @@
       <c r="AD12" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="AM12" t="s" s="0">
-        <v>292</v>
+      <c r="AM12" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="13" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>267</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>268</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>173</v>
@@ -3202,21 +3069,21 @@
         <v>171</v>
       </c>
       <c r="AC13" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AD13" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="AM13" t="s" s="0">
-        <v>292</v>
+      <c r="AM13" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="14" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>173</v>
@@ -3237,21 +3104,21 @@
         <v>177</v>
       </c>
       <c r="AC14" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="AD14" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="AD14" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="AM14" t="s" s="0">
-        <v>292</v>
+      <c r="AM14" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="15" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>173</v>
@@ -3272,13 +3139,13 @@
         <v>181</v>
       </c>
       <c r="AC15" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="AD15" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="AD15" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="AM15" t="s" s="0">
-        <v>292</v>
+      <c r="AM15" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -3297,13 +3164,13 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="11.6640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="18.33203125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="47.5546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.6640625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="21.109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.109375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="18.109375"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -3333,7 +3200,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -3354,8 +3221,8 @@
       <c r="G2" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="H2" t="s" s="0">
-        <v>292</v>
+      <c r="H2" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -3373,23 +3240,23 @@
   <dimension ref="A1:AP7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="11.44140625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="29.44140625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="82.33203125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.6640625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="21.109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="18.5546875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="14.33203125"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="13.88671875"/>
-    <col min="32" max="33" customWidth="true" width="13.88671875"/>
-    <col min="34" max="35" bestFit="true" customWidth="true" width="26.5546875"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="20.109375"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" width="15.6640625"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" width="21.88671875"/>
-    <col min="39" max="39" customWidth="true" width="21.88671875"/>
-    <col min="40" max="40" bestFit="true" customWidth="true" width="51.6640625"/>
-    <col min="41" max="41" bestFit="true" customWidth="true" width="11.0"/>
+    <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="82.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="13.88671875" customWidth="1"/>
+    <col min="34" max="35" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="21.88671875" customWidth="1"/>
+    <col min="40" max="40" width="51.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.3">
@@ -3521,7 +3388,7 @@
       </c>
     </row>
     <row r="2" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>106</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -3560,18 +3427,18 @@
       <c r="N2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AN2" t="s" s="0">
-        <v>306</v>
-      </c>
-      <c r="AO2" t="s" s="0">
-        <v>305</v>
-      </c>
-      <c r="AP2" t="s" s="0">
-        <v>292</v>
+      <c r="AN2" t="s">
+        <v>299</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>298</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>110</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -3620,23 +3487,23 @@
         <v>46</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="Z3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AN3" t="s" s="0">
-        <v>315</v>
-      </c>
-      <c r="AO3" t="s" s="0">
-        <v>314</v>
-      </c>
-      <c r="AP3" t="s" s="0">
-        <v>292</v>
+      <c r="AN3" t="s">
+        <v>324</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>323</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>113</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -3691,32 +3558,32 @@
         <v>52</v>
       </c>
       <c r="U4" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="V4" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="V4" s="3" t="s">
+      <c r="W4" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="W4" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="X4" s="3" t="s">
         <v>53</v>
       </c>
       <c r="Y4" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="AN4" t="s" s="0">
-        <v>308</v>
-      </c>
-      <c r="AO4" t="s" s="0">
-        <v>307</v>
-      </c>
-      <c r="AP4" t="s" s="0">
-        <v>292</v>
+        <v>284</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>326</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>325</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>115</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -3755,30 +3622,30 @@
       <c r="N5" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AJ5" s="0">
+      <c r="AJ5">
         <v>25</v>
       </c>
-      <c r="AK5" s="0">
-        <v>1918.2750000000001</v>
-      </c>
-      <c r="AL5" s="0">
-        <v>1918.2750000000001</v>
-      </c>
-      <c r="AM5" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="AN5" t="s" s="0">
-        <v>311</v>
-      </c>
-      <c r="AO5" t="s" s="0">
-        <v>309</v>
-      </c>
-      <c r="AP5" t="s" s="0">
-        <v>292</v>
+      <c r="AK5">
+        <v>2497.2469999999998</v>
+      </c>
+      <c r="AL5">
+        <v>2497.2469999999998</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>301</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>302</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>300</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>118</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -3827,32 +3694,32 @@
         <v>46</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="Z6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AM6" t="s" s="0">
-        <v>328</v>
-      </c>
-      <c r="AN6" t="s" s="0">
+      <c r="AM6" t="s">
+        <v>330</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>331</v>
+      </c>
+      <c r="AO6" t="s">
         <v>329</v>
       </c>
-      <c r="AO6" t="s" s="0">
-        <v>327</v>
-      </c>
-      <c r="AP6" t="s" s="0">
-        <v>292</v>
+      <c r="AP6" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>158</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="C7" t="s">
         <v>164</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -3895,34 +3762,34 @@
         <v>46</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="Z7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AE7" t="s" s="0">
+      <c r="AE7" t="s">
         <v>159</v>
       </c>
       <c r="AF7" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="AG7" s="0">
+      <c r="AG7">
         <v>0.4</v>
       </c>
-      <c r="AH7" s="0">
+      <c r="AH7">
         <v>20</v>
       </c>
-      <c r="AI7" s="0">
+      <c r="AI7">
         <v>24.6</v>
       </c>
-      <c r="AN7" t="s" s="0">
-        <v>326</v>
-      </c>
-      <c r="AO7" t="s" s="0">
-        <v>325</v>
-      </c>
-      <c r="AP7" t="s" s="0">
-        <v>292</v>
+      <c r="AN7" t="s">
+        <v>328</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>327</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -3950,21 +3817,21 @@
   <dimension ref="A1:Q25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="11.6640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="23.88671875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="123.6640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.6640625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="21.109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.109375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="19.88671875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.5546875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="36.109375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="18.33203125"/>
-    <col min="11" max="11" customWidth="true" width="18.0"/>
-    <col min="12" max="12" customWidth="true" width="18.33203125"/>
-    <col min="13" max="13" customWidth="true" width="14.5546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.6640625"/>
-    <col min="15" max="16" customWidth="true" width="14.5546875"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="123.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" customWidth="1"/>
+    <col min="13" max="13" width="14.5546875" customWidth="1"/>
+    <col min="14" max="14" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
@@ -4011,26 +3878,26 @@
         <v>224</v>
       </c>
       <c r="O1" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>253</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>254</v>
       </c>
       <c r="Q1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>123</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>137</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>124</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>65</v>
       </c>
       <c r="E2" s="3" t="s">
@@ -4039,30 +3906,30 @@
       <c r="F2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>125</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="H2" t="s">
         <v>125</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>126</v>
       </c>
-      <c r="Q2" t="s" s="0">
-        <v>292</v>
+      <c r="Q2" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>127</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>137</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>128</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>65</v>
       </c>
       <c r="E3" s="3" t="s">
@@ -4071,30 +3938,30 @@
       <c r="F3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" t="s" s="0">
+      <c r="G3" t="s">
         <v>129</v>
       </c>
-      <c r="H3" t="s" s="0">
+      <c r="H3" t="s">
         <v>130</v>
       </c>
-      <c r="I3" t="s" s="0">
+      <c r="I3" t="s">
         <v>131</v>
       </c>
-      <c r="Q3" t="s" s="0">
-        <v>292</v>
+      <c r="Q3" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>132</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>137</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>133</v>
       </c>
-      <c r="D4" t="s" s="0">
+      <c r="D4" t="s">
         <v>65</v>
       </c>
       <c r="E4" s="3" t="s">
@@ -4103,30 +3970,30 @@
       <c r="F4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G4" t="s" s="0">
+      <c r="G4" t="s">
         <v>134</v>
       </c>
-      <c r="H4" t="s" s="0">
+      <c r="H4" t="s">
         <v>135</v>
       </c>
-      <c r="I4" t="s" s="0">
+      <c r="I4" t="s">
         <v>136</v>
       </c>
-      <c r="Q4" t="s" s="0">
-        <v>292</v>
+      <c r="Q4" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>138</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>137</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s">
         <v>139</v>
       </c>
-      <c r="D5" t="s" s="0">
+      <c r="D5" t="s">
         <v>65</v>
       </c>
       <c r="E5" s="3" t="s">
@@ -4135,30 +4002,30 @@
       <c r="F5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G5" t="s" s="0">
+      <c r="G5" t="s">
         <v>140</v>
       </c>
-      <c r="H5" t="s" s="0">
+      <c r="H5" t="s">
         <v>141</v>
       </c>
-      <c r="I5" t="s" s="0">
+      <c r="I5" t="s">
         <v>142</v>
       </c>
-      <c r="Q5" t="s" s="0">
-        <v>292</v>
+      <c r="Q5" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>143</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>137</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="C6" t="s">
         <v>144</v>
       </c>
-      <c r="D6" t="s" s="0">
+      <c r="D6" t="s">
         <v>65</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -4167,30 +4034,30 @@
       <c r="F6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G6" t="s" s="0">
+      <c r="G6" t="s">
         <v>145</v>
       </c>
-      <c r="H6" t="s" s="0">
+      <c r="H6" t="s">
         <v>150</v>
       </c>
-      <c r="I6" t="s" s="0">
+      <c r="I6" t="s">
         <v>146</v>
       </c>
-      <c r="Q6" t="s" s="0">
-        <v>292</v>
+      <c r="Q6" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>147</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>137</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="C7" t="s">
         <v>148</v>
       </c>
-      <c r="D7" t="s" s="0">
+      <c r="D7" t="s">
         <v>65</v>
       </c>
       <c r="E7" s="3" t="s">
@@ -4199,30 +4066,30 @@
       <c r="F7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G7" t="s" s="0">
+      <c r="G7" t="s">
         <v>149</v>
       </c>
-      <c r="H7" t="s" s="0">
+      <c r="H7" t="s">
         <v>151</v>
       </c>
-      <c r="I7" t="s" s="0">
+      <c r="I7" t="s">
         <v>152</v>
       </c>
-      <c r="Q7" t="s" s="0">
-        <v>292</v>
+      <c r="Q7" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>153</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s">
         <v>137</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="C8" t="s">
         <v>154</v>
       </c>
-      <c r="D8" t="s" s="0">
+      <c r="D8" t="s">
         <v>65</v>
       </c>
       <c r="E8" s="3" t="s">
@@ -4231,30 +4098,30 @@
       <c r="F8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G8" t="s" s="0">
+      <c r="G8" t="s">
         <v>155</v>
       </c>
-      <c r="H8" t="s" s="0">
+      <c r="H8" t="s">
         <v>130</v>
       </c>
-      <c r="I8" t="s" s="0">
+      <c r="I8" t="s">
         <v>156</v>
       </c>
-      <c r="Q8" t="s" s="0">
-        <v>292</v>
+      <c r="Q8" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>185</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s">
         <v>137</v>
       </c>
-      <c r="C9" t="s" s="0">
+      <c r="C9" t="s">
         <v>186</v>
       </c>
-      <c r="D9" t="s" s="0">
+      <c r="D9" t="s">
         <v>65</v>
       </c>
       <c r="E9" s="3" t="s">
@@ -4263,30 +4130,30 @@
       <c r="F9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G9" t="s" s="0">
+      <c r="G9" t="s">
         <v>187</v>
       </c>
-      <c r="H9" t="s" s="0">
+      <c r="H9" t="s">
         <v>188</v>
       </c>
-      <c r="I9" t="s" s="0">
+      <c r="I9" t="s">
         <v>189</v>
       </c>
-      <c r="Q9" t="s" s="0">
-        <v>292</v>
+      <c r="Q9" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>196</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="B10" t="s">
         <v>230</v>
       </c>
-      <c r="C10" t="s" s="0">
+      <c r="C10" t="s">
         <v>197</v>
       </c>
-      <c r="D10" t="s" s="0">
+      <c r="D10" t="s">
         <v>65</v>
       </c>
       <c r="E10" s="3" t="s">
@@ -4295,27 +4162,27 @@
       <c r="F10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G10" t="s" s="0">
+      <c r="G10" t="s">
         <v>202</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="Q10" t="s" s="0">
-        <v>292</v>
+      <c r="Q10" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>203</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="B11" t="s">
         <v>230</v>
       </c>
-      <c r="C11" t="s" s="0">
+      <c r="C11" t="s">
         <v>204</v>
       </c>
-      <c r="D11" t="s" s="0">
+      <c r="D11" t="s">
         <v>65</v>
       </c>
       <c r="E11" s="3" t="s">
@@ -4324,27 +4191,27 @@
       <c r="F11" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G11" t="s" s="0">
+      <c r="G11" t="s">
         <v>205</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="Q11" t="s" s="0">
-        <v>292</v>
+        <v>304</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A12" t="s" s="0">
+      <c r="A12" t="s">
         <v>206</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="B12" t="s">
         <v>230</v>
       </c>
-      <c r="C12" t="s" s="0">
+      <c r="C12" t="s">
         <v>207</v>
       </c>
-      <c r="D12" t="s" s="0">
+      <c r="D12" t="s">
         <v>65</v>
       </c>
       <c r="E12" s="3" t="s">
@@ -4353,27 +4220,27 @@
       <c r="F12" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G12" t="s" s="0">
+      <c r="G12" t="s">
         <v>208</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="Q12" t="s" s="0">
-        <v>292</v>
+      <c r="Q12" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A13" t="s" s="0">
+      <c r="A13" t="s">
         <v>210</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="B13" t="s">
         <v>230</v>
       </c>
-      <c r="C13" t="s" s="0">
+      <c r="C13" t="s">
         <v>211</v>
       </c>
-      <c r="D13" t="s" s="0">
+      <c r="D13" t="s">
         <v>65</v>
       </c>
       <c r="E13" s="3" t="s">
@@ -4382,27 +4249,27 @@
       <c r="F13" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G13" t="s" s="0">
+      <c r="G13" t="s">
         <v>151</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>291</v>
-      </c>
-      <c r="Q13" t="s" s="0">
-        <v>292</v>
+        <v>305</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A14" t="s" s="0">
+      <c r="A14" t="s">
         <v>212</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="B14" t="s">
         <v>230</v>
       </c>
-      <c r="C14" t="s" s="0">
+      <c r="C14" t="s">
         <v>213</v>
       </c>
-      <c r="D14" t="s" s="0">
+      <c r="D14" t="s">
         <v>65</v>
       </c>
       <c r="E14" s="3" t="s">
@@ -4411,27 +4278,27 @@
       <c r="F14" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G14" t="s" s="0">
+      <c r="G14" t="s">
         <v>214</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="Q14" t="s" s="0">
-        <v>292</v>
+      <c r="Q14" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A15" t="s" s="0">
+      <c r="A15" t="s">
         <v>216</v>
       </c>
-      <c r="B15" t="s" s="0">
+      <c r="B15" t="s">
         <v>230</v>
       </c>
-      <c r="C15" t="s" s="0">
+      <c r="C15" t="s">
         <v>217</v>
       </c>
-      <c r="D15" t="s" s="0">
+      <c r="D15" t="s">
         <v>65</v>
       </c>
       <c r="E15" s="3" t="s">
@@ -4440,27 +4307,27 @@
       <c r="F15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G15" t="s" s="0">
+      <c r="G15" t="s">
         <v>218</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="Q15" t="s" s="0">
-        <v>292</v>
+      <c r="Q15" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A16" t="s" s="0">
+      <c r="A16" t="s">
         <v>219</v>
       </c>
-      <c r="B16" t="s" s="0">
+      <c r="B16" t="s">
         <v>230</v>
       </c>
-      <c r="C16" t="s" s="0">
+      <c r="C16" t="s">
         <v>220</v>
       </c>
-      <c r="D16" t="s" s="0">
+      <c r="D16" t="s">
         <v>65</v>
       </c>
       <c r="E16" s="3" t="s">
@@ -4469,56 +4336,56 @@
       <c r="F16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G16" t="s" s="0">
+      <c r="G16" t="s">
         <v>221</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="Q16" t="s" s="0">
-        <v>292</v>
+      <c r="Q16" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A17" t="s" s="0">
+      <c r="A17" t="s">
+        <v>262</v>
+      </c>
+      <c r="B17" t="s">
+        <v>230</v>
+      </c>
+      <c r="C17" t="s">
         <v>263</v>
       </c>
-      <c r="B17" t="s" s="0">
-        <v>230</v>
-      </c>
-      <c r="C17" t="s" s="0">
+      <c r="D17" t="s">
+        <v>65</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G17" t="s">
+        <v>244</v>
+      </c>
+      <c r="I17" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="D17" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G17" t="s" s="0">
-        <v>245</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="Q17" t="s" s="0">
-        <v>292</v>
+      <c r="Q17" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18" t="s" s="0">
+      <c r="A18" t="s">
         <v>225</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="B18" t="s">
         <v>231</v>
       </c>
-      <c r="C18" t="s" s="0">
+      <c r="C18" t="s">
         <v>226</v>
       </c>
-      <c r="D18" t="s" s="0">
+      <c r="D18" t="s">
         <v>65</v>
       </c>
       <c r="E18" s="3" t="s">
@@ -4527,36 +4394,36 @@
       <c r="F18" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G18" t="s" s="0">
+      <c r="G18" t="s">
         <v>221</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="J18" t="s" s="0">
+      <c r="J18" t="s">
         <v>228</v>
       </c>
-      <c r="L18" t="s" s="0">
+      <c r="L18" t="s">
         <v>178</v>
       </c>
-      <c r="N18" t="s" s="0">
+      <c r="N18" t="s">
         <v>229</v>
       </c>
-      <c r="Q18" t="s" s="0">
-        <v>292</v>
+      <c r="Q18" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A19" t="s" s="0">
+      <c r="A19" t="s">
         <v>232</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="B19" t="s">
         <v>231</v>
       </c>
-      <c r="C19" t="s" s="0">
+      <c r="C19" t="s">
         <v>233</v>
       </c>
-      <c r="D19" t="s" s="0">
+      <c r="D19" t="s">
         <v>65</v>
       </c>
       <c r="E19" s="3" t="s">
@@ -4565,36 +4432,36 @@
       <c r="F19" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G19" t="s" s="0">
+      <c r="G19" t="s">
         <v>202</v>
       </c>
       <c r="I19" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="J19" t="s">
+        <v>234</v>
+      </c>
+      <c r="K19" t="s">
+        <v>235</v>
+      </c>
+      <c r="L19" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>236</v>
       </c>
-      <c r="J19" t="s" s="0">
-        <v>234</v>
-      </c>
-      <c r="K19" t="s" s="0">
-        <v>235</v>
-      </c>
-      <c r="L19" t="s" s="0">
-        <v>178</v>
-      </c>
-      <c r="Q19" t="s" s="0">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A20" t="s" s="0">
+      <c r="B20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C20" t="s">
         <v>237</v>
       </c>
-      <c r="B20" t="s" s="0">
-        <v>231</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>238</v>
-      </c>
-      <c r="D20" t="s" s="0">
+      <c r="D20" t="s">
         <v>65</v>
       </c>
       <c r="E20" s="3" t="s">
@@ -4603,210 +4470,210 @@
       <c r="F20" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G20" t="s" s="0">
+      <c r="G20" t="s">
         <v>205</v>
       </c>
       <c r="I20" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="J20" t="s" s="0">
+      <c r="J20" t="s">
+        <v>238</v>
+      </c>
+      <c r="L20" t="s">
+        <v>178</v>
+      </c>
+      <c r="N20" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>239</v>
       </c>
-      <c r="L20" t="s" s="0">
+      <c r="B21" t="s">
+        <v>231</v>
+      </c>
+      <c r="C21" t="s">
+        <v>240</v>
+      </c>
+      <c r="D21" t="s">
+        <v>65</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" t="s">
+        <v>208</v>
+      </c>
+      <c r="J21" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>243</v>
+      </c>
+      <c r="B22" t="s">
+        <v>231</v>
+      </c>
+      <c r="C22" t="s">
+        <v>242</v>
+      </c>
+      <c r="D22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G22" t="s">
+        <v>244</v>
+      </c>
+      <c r="I22" t="s">
+        <v>245</v>
+      </c>
+      <c r="J22" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>246</v>
+      </c>
+      <c r="B23" t="s">
+        <v>231</v>
+      </c>
+      <c r="C23" t="s">
+        <v>247</v>
+      </c>
+      <c r="D23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I23" t="s">
+        <v>303</v>
+      </c>
+      <c r="J23" t="s">
+        <v>289</v>
+      </c>
+      <c r="K23" t="s">
+        <v>235</v>
+      </c>
+      <c r="L23" t="s">
         <v>178</v>
       </c>
-      <c r="N20" t="s" s="0">
+      <c r="Q23" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>248</v>
+      </c>
+      <c r="B24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C24" t="s">
+        <v>249</v>
+      </c>
+      <c r="D24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G24" t="s">
+        <v>214</v>
+      </c>
+      <c r="I24" t="s">
+        <v>256</v>
+      </c>
+      <c r="J24" t="s">
+        <v>250</v>
+      </c>
+      <c r="L24" t="s">
+        <v>251</v>
+      </c>
+      <c r="N24" t="s">
         <v>229</v>
       </c>
-      <c r="Q20" t="s" s="0">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A21" t="s" s="0">
-        <v>240</v>
-      </c>
-      <c r="B21" t="s" s="0">
+      <c r="O24" t="s">
+        <v>254</v>
+      </c>
+      <c r="P24" t="s">
+        <v>255</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>257</v>
+      </c>
+      <c r="B25" t="s">
         <v>231</v>
       </c>
-      <c r="C21" t="s" s="0">
-        <v>241</v>
-      </c>
-      <c r="D21" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G21" t="s" s="0">
-        <v>208</v>
-      </c>
-      <c r="J21" t="s" s="0">
-        <v>242</v>
-      </c>
-      <c r="Q21" t="s" s="0">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A22" t="s" s="0">
-        <v>244</v>
-      </c>
-      <c r="B22" t="s" s="0">
-        <v>231</v>
-      </c>
-      <c r="C22" t="s" s="0">
-        <v>243</v>
-      </c>
-      <c r="D22" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G22" t="s" s="0">
-        <v>245</v>
-      </c>
-      <c r="I22" t="s" s="0">
-        <v>246</v>
-      </c>
-      <c r="J22" t="s" s="0">
-        <v>130</v>
-      </c>
-      <c r="Q22" t="s" s="0">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A23" t="s" s="0">
-        <v>247</v>
-      </c>
-      <c r="B23" t="s" s="0">
-        <v>231</v>
-      </c>
-      <c r="C23" t="s" s="0">
-        <v>248</v>
-      </c>
-      <c r="D23" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G23" t="s" s="0">
-        <v>151</v>
-      </c>
-      <c r="I23" t="s" s="0">
-        <v>313</v>
-      </c>
-      <c r="J23" t="s" s="0">
-        <v>312</v>
-      </c>
-      <c r="K23" t="s" s="0">
-        <v>235</v>
-      </c>
-      <c r="L23" t="s" s="0">
-        <v>178</v>
-      </c>
-      <c r="Q23" t="s" s="0">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A24" t="s" s="0">
-        <v>249</v>
-      </c>
-      <c r="B24" t="s" s="0">
-        <v>231</v>
-      </c>
-      <c r="C24" t="s" s="0">
-        <v>250</v>
-      </c>
-      <c r="D24" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G24" t="s" s="0">
-        <v>214</v>
-      </c>
-      <c r="I24" t="s" s="0">
-        <v>257</v>
-      </c>
-      <c r="J24" t="s" s="0">
+      <c r="C25" t="s">
+        <v>258</v>
+      </c>
+      <c r="D25" t="s">
+        <v>65</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G25" t="s">
+        <v>218</v>
+      </c>
+      <c r="I25" t="s">
+        <v>261</v>
+      </c>
+      <c r="J25" t="s">
+        <v>259</v>
+      </c>
+      <c r="L25" t="s">
         <v>251</v>
       </c>
-      <c r="L24" t="s" s="0">
-        <v>252</v>
-      </c>
-      <c r="N24" t="s" s="0">
-        <v>229</v>
-      </c>
-      <c r="O24" t="s" s="0">
+      <c r="N25" t="s">
+        <v>260</v>
+      </c>
+      <c r="O25" t="s">
+        <v>254</v>
+      </c>
+      <c r="P25" t="s">
         <v>255</v>
       </c>
-      <c r="P24" t="s" s="0">
-        <v>256</v>
-      </c>
-      <c r="Q24" t="s" s="0">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A25" t="s" s="0">
-        <v>258</v>
-      </c>
-      <c r="B25" t="s" s="0">
-        <v>231</v>
-      </c>
-      <c r="C25" t="s" s="0">
-        <v>259</v>
-      </c>
-      <c r="D25" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G25" t="s" s="0">
-        <v>218</v>
-      </c>
-      <c r="I25" t="s" s="0">
-        <v>262</v>
-      </c>
-      <c r="J25" t="s" s="0">
-        <v>260</v>
-      </c>
-      <c r="L25" t="s" s="0">
-        <v>252</v>
-      </c>
-      <c r="N25" t="s" s="0">
-        <v>261</v>
-      </c>
-      <c r="O25" t="s" s="0">
-        <v>255</v>
-      </c>
-      <c r="P25" t="s" s="0">
-        <v>256</v>
-      </c>
-      <c r="Q25" t="s" s="0">
-        <v>292</v>
+      <c r="Q25" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -4831,15 +4698,15 @@
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.44140625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="14.33203125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="47.5546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.6640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.109375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="18.109375"/>
-    <col min="9" max="9" customWidth="true" width="18.109375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" customWidth="1"/>
+    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -4865,51 +4732,51 @@
         <v>7</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>277</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>278</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>284</v>
-      </c>
       <c r="H2" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="J2" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="K2" t="s" s="0">
-        <v>292</v>
+      <c r="K2" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>